<commit_message>
Commit remaining plugin updates
</commit_message>
<xml_diff>
--- a/MH_Registry/superimp_library.xlsx
+++ b/MH_Registry/superimp_library.xlsx
@@ -2797,12 +2797,29 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
+          <t xml:space="preserve">HDFCA.DONGWA</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">9</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
           <t xml:space="preserve">GOTN</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">9</t>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(registry): activate DC thickness bindings immediately
</commit_message>
<xml_diff>
--- a/MH_Registry/superimp_library.xlsx
+++ b/MH_Registry/superimp_library.xlsx
@@ -4,11 +4,10 @@
   <sheets>
     <sheet name="superimp_import_list" sheetId="1" r:id="rId1"/>
     <sheet name="dc_manual_materials" sheetId="2" r:id="rId2"/>
-    <sheet name="dc_thickness_options" sheetId="3" r:id="rId3"/>
-    <sheet name="dc_thickness_bindings" sheetId="4" r:id="rId4"/>
-    <sheet name="dc_material_profiles" sheetId="5" r:id="rId5"/>
-    <sheet name="dc_material_options" sheetId="6" r:id="rId6"/>
-    <sheet name="material_profile_choices" sheetId="7" r:id="rId7"/>
+    <sheet name="dc_thickness_bindings" sheetId="3" r:id="rId3"/>
+    <sheet name="dc_material_profiles" sheetId="4" r:id="rId4"/>
+    <sheet name="dc_material_options" sheetId="5" r:id="rId5"/>
+    <sheet name="material_profile_choices" sheetId="6" r:id="rId6"/>
   </sheets>
 </workbook>
 </file>
@@ -2656,187 +2655,522 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve">1</t>
+          <t xml:space="preserve">0</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t xml:space="preserve">PLY</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1</t>
-        </is>
-      </c>
+          <t xml:space="preserve">GOGT</t>
+        </is>
+      </c>
+      <c r="C2"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1</t>
+          <t xml:space="preserve">0</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t xml:space="preserve">HDFCA.AC</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2</t>
-        </is>
-      </c>
+          <t xml:space="preserve">GONHUA</t>
+        </is>
+      </c>
+      <c r="C3"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve">1</t>
+          <t xml:space="preserve">0</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t xml:space="preserve">HDFCA.AC.LK</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">3</t>
-        </is>
-      </c>
+          <t xml:space="preserve">GOSOI</t>
+        </is>
+      </c>
+      <c r="C4"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t xml:space="preserve">1</t>
+          <t xml:space="preserve">0</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t xml:space="preserve">GOSOI</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">4</t>
-        </is>
-      </c>
+          <t xml:space="preserve">GOTN</t>
+        </is>
+      </c>
+      <c r="C5"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">1</t>
+          <t xml:space="preserve">0</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t xml:space="preserve">PLY.AC.VERSOI</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">5</t>
-        </is>
-      </c>
+          <t xml:space="preserve">HDFCA.AC</t>
+        </is>
+      </c>
+      <c r="C6"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">1</t>
+          <t xml:space="preserve">0</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t xml:space="preserve">WPB</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">6</t>
-        </is>
-      </c>
+          <t xml:space="preserve">HDFCA.AC.LK</t>
+        </is>
+      </c>
+      <c r="C7"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">1</t>
+          <t xml:space="preserve">0</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t xml:space="preserve">PLY.AC</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">7</t>
-        </is>
-      </c>
+          <t xml:space="preserve">HDFCA.AC.MS</t>
+        </is>
+      </c>
+      <c r="C8"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">1</t>
+          <t xml:space="preserve">0</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t xml:space="preserve">PICOMAT</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">8</t>
-        </is>
-      </c>
+          <t xml:space="preserve">HDFCA.AC.VER</t>
+        </is>
+      </c>
+      <c r="C9"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve">1</t>
+          <t xml:space="preserve">0</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t xml:space="preserve">GOGT</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">9</t>
-        </is>
-      </c>
+          <t xml:space="preserve">HDFCA.AC.VERSOI</t>
+        </is>
+      </c>
+      <c r="C10"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve">1</t>
+          <t xml:space="preserve">0</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t xml:space="preserve">HDFCA.DONGWA</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">10</t>
-        </is>
-      </c>
+          <t xml:space="preserve">HDFCA.DW</t>
+        </is>
+      </c>
+      <c r="C11"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">1</t>
+          <t xml:space="preserve">0</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t xml:space="preserve">GOTN</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">11</t>
+          <t xml:space="preserve">HDFCA.DW.LK</t>
+        </is>
+      </c>
+      <c r="C12"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HDFCA.DW.VANDA</t>
+        </is>
+      </c>
+      <c r="C13"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MDFCA.AC.LAM</t>
+        </is>
+      </c>
+      <c r="C14"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MDFCA.AC.MEL</t>
+        </is>
+      </c>
+      <c r="C15"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MDFCA.PANEL</t>
+        </is>
+      </c>
+      <c r="C16"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MDFCA.PANEL.VERTANBI</t>
+        </is>
+      </c>
+      <c r="C17"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PICOMAT</t>
+        </is>
+      </c>
+      <c r="C18"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PLY</t>
+        </is>
+      </c>
+      <c r="C19"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PLY.AC</t>
+        </is>
+      </c>
+      <c r="C20"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PLY.AC.LK</t>
+        </is>
+      </c>
+      <c r="C21"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PLY.AC.MS</t>
+        </is>
+      </c>
+      <c r="C22"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PLY.AC.VER</t>
+        </is>
+      </c>
+      <c r="C23"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PLY.AC.VERKTSOI</t>
+        </is>
+      </c>
+      <c r="C24"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PLY.AC.VERSOI</t>
+        </is>
+      </c>
+      <c r="C25"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PLY.LK</t>
+        </is>
+      </c>
+      <c r="C26"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PLY.VANDA</t>
+        </is>
+      </c>
+      <c r="C27"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PLY.VER</t>
+        </is>
+      </c>
+      <c r="C28"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TANBI</t>
+        </is>
+      </c>
+      <c r="C29"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WPB</t>
+        </is>
+      </c>
+      <c r="C30"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WPB.LAM</t>
+        </is>
+      </c>
+      <c r="C31"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WPB.LK</t>
+        </is>
+      </c>
+      <c r="C32"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MDFCA.ML.MEL.ML5009SMM</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MDFCA.ML.MEL.ML6325</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PLY.17.E0.AC</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MDFCA.17.E1.TL</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MDFCA.E1.AC.SON</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MDFCA.AC.SON</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GGT</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">7</t>
         </is>
       </c>
     </row>
@@ -2850,1043 +3184,1001 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t xml:space="preserve">material_type</t>
+          <t xml:space="preserve">match</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t xml:space="preserve">opt1_panel</t>
+          <t xml:space="preserve">label</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t xml:space="preserve">opt1_back</t>
+          <t xml:space="preserve">param_panel</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t xml:space="preserve">opt2_panel</t>
+          <t xml:space="preserve">param_back</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t xml:space="preserve">opt2_back</t>
+          <t xml:space="preserve">param_extra</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t xml:space="preserve">opt3_panel</t>
+          <t xml:space="preserve">product_only</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t xml:space="preserve">opt3_back</t>
+          <t xml:space="preserve">unit</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t xml:space="preserve">opt4_panel</t>
+          <t xml:space="preserve">enabled</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t xml:space="preserve">opt4_back</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">opt5_panel</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">opt5_back</t>
+          <t xml:space="preserve">modul_only</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve">GOGT</t>
+          <t xml:space="preserve">Tấm fix</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t xml:space="preserve">20</t>
-        </is>
-      </c>
-      <c r="C2"/>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">26</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Độ dày</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">definition:d1</t>
+        </is>
+      </c>
+      <c r="D2"/>
       <c r="E2"/>
       <c r="F2"/>
-      <c r="G2"/>
-      <c r="H2"/>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mm</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
       <c r="I2"/>
-      <c r="J2"/>
-      <c r="K2"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t xml:space="preserve">GONHUA</t>
+          <t xml:space="preserve">Ngắn Kéo Đáy Lùa</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t xml:space="preserve">17.6</t>
+          <t xml:space="preserve">Panel: Độ Dày Tấm Panel Thickness | Hậu: Đáy - Độ Dày Tấm Bottom Thickness</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t xml:space="preserve">10</t>
+          <t xml:space="preserve">definition:eqgyit1tf1</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t xml:space="preserve">17.6</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">11</t>
-        </is>
-      </c>
+          <t xml:space="preserve">definition:erhqw_82nd</t>
+        </is>
+      </c>
+      <c r="E3"/>
       <c r="F3"/>
-      <c r="G3"/>
-      <c r="H3"/>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mm</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
       <c r="I3"/>
-      <c r="J3"/>
-      <c r="K3"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve">GONHUA.AC</t>
+          <t xml:space="preserve">Khung Tủ Lạnh</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t xml:space="preserve">17.6</t>
+          <t xml:space="preserve">Độ Dày Tấm Panel Thickness, Hậu Độ Dày Tấm Back Thickness</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t xml:space="preserve">10</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">17.6</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">11</t>
-        </is>
-      </c>
+          <t xml:space="preserve">definition:ba4ulq2qnw, definition:ikqikbwfw7</t>
+        </is>
+      </c>
+      <c r="D4"/>
+      <c r="E4"/>
       <c r="F4"/>
-      <c r="G4"/>
-      <c r="H4"/>
-      <c r="I4"/>
-      <c r="J4"/>
-      <c r="K4"/>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mm</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t xml:space="preserve">GOSOI</t>
+          <t xml:space="preserve">Khung Nóc Lọt</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t xml:space="preserve">20</t>
-        </is>
-      </c>
-      <c r="C5"/>
+          <t xml:space="preserve">Panel: Độ Dày Tấm Panel Thickness | Hậu: Hậu Độ Dày Tấm Back Thickness</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">definition:ba4ulq2qnw</t>
+        </is>
+      </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t xml:space="preserve">26</t>
+          <t xml:space="preserve">definition:ikqikbwfw7</t>
         </is>
       </c>
       <c r="E5"/>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">38</t>
-        </is>
-      </c>
-      <c r="G5"/>
+      <c r="F5"/>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mm</t>
+        </is>
+      </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t xml:space="preserve">50</t>
-        </is>
-      </c>
-      <c r="I5"/>
-      <c r="J5"/>
-      <c r="K5"/>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">GOTN</t>
+          <t xml:space="preserve">Khung Bếp 1</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t xml:space="preserve">20</t>
-        </is>
-      </c>
-      <c r="C6"/>
+          <t xml:space="preserve">Panel: Độ Dày Tấm Panel Thickness | Hậu: Hậu Độ Dày Tấm Back Thickness</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">definition:abh13iq2kv</t>
+        </is>
+      </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t xml:space="preserve">26</t>
+          <t xml:space="preserve">definition:g3dnsrlh5l</t>
         </is>
       </c>
       <c r="E6"/>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">32</t>
-        </is>
-      </c>
-      <c r="G6"/>
-      <c r="H6"/>
-      <c r="I6"/>
-      <c r="J6"/>
-      <c r="K6"/>
+      <c r="F6"/>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">length</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">HDFCA.AC</t>
+          <t xml:space="preserve">Ngăn kéo ray bi</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t xml:space="preserve">17.6</t>
+          <t xml:space="preserve">Panel: Độ Dày Tấm Panel Thickness | Hậu: Đáy - Độ Dày Tấm Bottom Thickness</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t xml:space="preserve">11</t>
+          <t xml:space="preserve">definition:eqgyit1tf1</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t xml:space="preserve">17.6</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">8</t>
-        </is>
-      </c>
+          <t xml:space="preserve">definition:erhqw_82nd</t>
+        </is>
+      </c>
+      <c r="E7"/>
       <c r="F7"/>
-      <c r="G7"/>
-      <c r="H7"/>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mm</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
       <c r="I7"/>
-      <c r="J7"/>
-      <c r="K7"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">HDFCA.AC.LK</t>
+          <t xml:space="preserve">Đáy</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t xml:space="preserve">19.6</t>
+          <t xml:space="preserve">Chiều dày ván</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t xml:space="preserve">11</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">19.6</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">8</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">19.6</t>
-        </is>
-      </c>
+          <t xml:space="preserve">definition:d1</t>
+        </is>
+      </c>
+      <c r="D8"/>
+      <c r="E8"/>
+      <c r="F8"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t xml:space="preserve">10</t>
+          <t xml:space="preserve">mm</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t xml:space="preserve">14</t>
+          <t xml:space="preserve">1</t>
         </is>
       </c>
       <c r="I8"/>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">11</t>
-        </is>
-      </c>
-      <c r="K8"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">HDFCA.AC.MS</t>
+          <t xml:space="preserve">Nẹp Bù Trái 17</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t xml:space="preserve">17.6</t>
+          <t xml:space="preserve">Độ dày tấm</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t xml:space="preserve">11</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">17.6</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">8</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">17.6</t>
-        </is>
-      </c>
+          <t xml:space="preserve">definition:d1</t>
+        </is>
+      </c>
+      <c r="D9"/>
+      <c r="E9"/>
+      <c r="F9"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t xml:space="preserve">17.6</t>
-        </is>
-      </c>
-      <c r="H9"/>
+          <t xml:space="preserve">mm</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
       <c r="I9"/>
-      <c r="J9"/>
-      <c r="K9"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve">HDFCA.AC.VER</t>
+          <t xml:space="preserve">Nẹp Bù Phải 17</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t xml:space="preserve">18.6</t>
+          <t xml:space="preserve">Độ dày tấm</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t xml:space="preserve">10</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">18.6</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">8</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">11</t>
-        </is>
-      </c>
+          <t xml:space="preserve">definition:d1</t>
+        </is>
+      </c>
+      <c r="D10"/>
+      <c r="E10"/>
+      <c r="F10"/>
       <c r="G10" t="inlineStr">
         <is>
-          <t xml:space="preserve">0</t>
-        </is>
-      </c>
-      <c r="H10"/>
+          <t xml:space="preserve">mm</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
       <c r="I10"/>
-      <c r="J10"/>
-      <c r="K10"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve">HDFCA.AC.VERSOI</t>
+          <t xml:space="preserve">Nẹp Bù Phải 50</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t xml:space="preserve">18.6</t>
+          <t xml:space="preserve">Độ Dày Tấm</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t xml:space="preserve">10</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">18.6</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">8</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">14</t>
-        </is>
-      </c>
-      <c r="G11"/>
+          <t xml:space="preserve">definition:dodaytam</t>
+        </is>
+      </c>
+      <c r="D11"/>
+      <c r="E11"/>
+      <c r="F11"/>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mm</t>
+        </is>
+      </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t xml:space="preserve">18.6</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">18.6</t>
-        </is>
-      </c>
-      <c r="J11"/>
-      <c r="K11"/>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
+      <c r="I11"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">HDFCA.DONGWA</t>
+          <t xml:space="preserve">Nẹp Bù Trái 50</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t xml:space="preserve">17.6</t>
+          <t xml:space="preserve">Độ Dày Tấm</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t xml:space="preserve">10</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">17.6</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">11</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">17.6</t>
-        </is>
-      </c>
+          <t xml:space="preserve">definition:dodaytam</t>
+        </is>
+      </c>
+      <c r="D12"/>
+      <c r="E12"/>
+      <c r="F12"/>
       <c r="G12" t="inlineStr">
         <is>
-          <t xml:space="preserve">17.6</t>
-        </is>
-      </c>
-      <c r="H12"/>
+          <t xml:space="preserve">mm</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
       <c r="I12"/>
-      <c r="J12"/>
-      <c r="K12"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">HDFCA.DONGWA.LK</t>
+          <t xml:space="preserve">Đợt Cố Định</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t xml:space="preserve">18.6</t>
+          <t xml:space="preserve">Chiều dày ván</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t xml:space="preserve">10</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">18.6</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">18.6</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">14</t>
-        </is>
-      </c>
-      <c r="G13"/>
-      <c r="H13"/>
+          <t xml:space="preserve">definition:d1</t>
+        </is>
+      </c>
+      <c r="D13"/>
+      <c r="E13"/>
+      <c r="F13"/>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mm</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
       <c r="I13"/>
-      <c r="J13"/>
-      <c r="K13"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">HDFCA.DONGWA.VANDA</t>
+          <t xml:space="preserve">Khung lavabo 1</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t xml:space="preserve">18.6</t>
+          <t xml:space="preserve">Độ Dày Tấm Panel Thickness, Hậu Độ Dày Tấm Back Thickness</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t xml:space="preserve">10</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">18.6</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">18.6</t>
-        </is>
-      </c>
+          <t xml:space="preserve">definition:ba4ulq2qnw, definition:ikqikbwfw7</t>
+        </is>
+      </c>
+      <c r="D14"/>
+      <c r="E14"/>
       <c r="F14"/>
-      <c r="G14"/>
-      <c r="H14"/>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mm</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
       <c r="I14"/>
-      <c r="J14"/>
-      <c r="K14"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve">MDFCA.PANEL</t>
+          <t xml:space="preserve">Phào Nóc</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t xml:space="preserve">17.6</t>
+          <t xml:space="preserve">Độ Dày Tấm</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t xml:space="preserve">8</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">17.6</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">11</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">17.6</t>
-        </is>
-      </c>
+          <t xml:space="preserve">definition:ddaytam</t>
+        </is>
+      </c>
+      <c r="D15"/>
+      <c r="E15"/>
+      <c r="F15"/>
       <c r="G15" t="inlineStr">
         <is>
-          <t xml:space="preserve">17.6</t>
-        </is>
-      </c>
-      <c r="H15"/>
+          <t xml:space="preserve">mm</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
       <c r="I15"/>
-      <c r="J15"/>
-      <c r="K15"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t xml:space="preserve">MDFCA.PANEL.VERTANBI</t>
+          <t xml:space="preserve">Ngăn Kéo Ray Âm</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t xml:space="preserve">18.6</t>
+          <t xml:space="preserve">Panel: Độ Dày Tấm Panel Thickness | Hậu: Đáy - Độ Dày Tấm Bottom Thickness</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t xml:space="preserve">11</t>
+          <t xml:space="preserve">definition:eqgyit1tf1</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t xml:space="preserve">18.6</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">8</t>
-        </is>
-      </c>
+          <t xml:space="preserve">definition:erhqw_82nd</t>
+        </is>
+      </c>
+      <c r="E16"/>
       <c r="F16"/>
-      <c r="G16"/>
-      <c r="H16"/>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mm</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
       <c r="I16"/>
-      <c r="J16"/>
-      <c r="K16"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t xml:space="preserve">PICOMAT</t>
+          <t xml:space="preserve">Cánh Pano</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t xml:space="preserve">18.6</t>
+          <t xml:space="preserve">Panel: Độ Dày Ván | Hậu: Chiều Rộng Rãnh Soi</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t xml:space="preserve">10</t>
-        </is>
-      </c>
-      <c r="D17"/>
+          <t xml:space="preserve">definition:a0van</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">definition:c1</t>
+        </is>
+      </c>
       <c r="E17"/>
       <c r="F17"/>
-      <c r="G17"/>
-      <c r="H17"/>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mm</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
       <c r="I17"/>
-      <c r="J17"/>
-      <c r="K17"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">PLY</t>
+          <t xml:space="preserve">Khung Nóc Phủ</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t xml:space="preserve">17.6</t>
+          <t xml:space="preserve">Panel: Độ Dày Tấm Panel Thickness | Hậu: Hậu Độ Dày Tấm Back Thickness</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t xml:space="preserve">8</t>
+          <t xml:space="preserve">definition:blcep_e9zm</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t xml:space="preserve">17.6</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">11</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">17.6</t>
-        </is>
-      </c>
+          <t xml:space="preserve">definition:j3vpfsl6fq</t>
+        </is>
+      </c>
+      <c r="E18"/>
+      <c r="F18"/>
       <c r="G18" t="inlineStr">
         <is>
-          <t xml:space="preserve">17.6</t>
-        </is>
-      </c>
-      <c r="H18"/>
-      <c r="I18"/>
-      <c r="J18"/>
-      <c r="K18"/>
+          <t xml:space="preserve">length</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve">PLY.AC</t>
+          <t xml:space="preserve">Khung Nóc Phủ 100</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t xml:space="preserve">17.6</t>
+          <t xml:space="preserve">Panel: Độ Dày Tấm Panel Thickness | Hậu: Hậu Độ Dày Tấm Back Thickness</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t xml:space="preserve">11</t>
-        </is>
-      </c>
-      <c r="D19"/>
+          <t xml:space="preserve">definition:blcep_e9zm</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">definition:j3vpfsl6fq</t>
+        </is>
+      </c>
       <c r="E19"/>
       <c r="F19"/>
-      <c r="G19"/>
-      <c r="H19"/>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">length</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
       <c r="I19"/>
-      <c r="J19"/>
-      <c r="K19"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t xml:space="preserve">PLY.AC.LK</t>
+          <t xml:space="preserve">Chân Bệ</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t xml:space="preserve">18.6</t>
+          <t xml:space="preserve">độ dày ván</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t xml:space="preserve">11</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">18.6</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">8</t>
-        </is>
-      </c>
+          <t xml:space="preserve">definition:a5dodayvan</t>
+        </is>
+      </c>
+      <c r="D20"/>
+      <c r="E20"/>
       <c r="F20"/>
-      <c r="G20"/>
-      <c r="H20"/>
-      <c r="I20"/>
-      <c r="J20"/>
-      <c r="K20"/>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mm</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t xml:space="preserve">PLY.AC.MS</t>
+          <t xml:space="preserve">Ngăn Kéo Ray Âm 550</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t xml:space="preserve">17.6</t>
+          <t xml:space="preserve">Panel: Độ Dày Tấm Panel Thickness | Hậu: Đáy - Độ Dày Tấm Bottom Thickness</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t xml:space="preserve">11</t>
+          <t xml:space="preserve">definition:eqgyit1tf1</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t xml:space="preserve">17.6</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">17.6</t>
-        </is>
-      </c>
+          <t xml:space="preserve">definition:erhqw_82nd</t>
+        </is>
+      </c>
+      <c r="E21"/>
       <c r="F21"/>
-      <c r="G21"/>
-      <c r="H21"/>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">length</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
       <c r="I21"/>
-      <c r="J21"/>
-      <c r="K21"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t xml:space="preserve">PLY.AC.VER</t>
+          <t xml:space="preserve">Ngăn Kéo Ray Âm 500</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t xml:space="preserve">18.6</t>
+          <t xml:space="preserve">Panel: Độ Dày Tấm Panel Thickness | Hậu: Đáy - Độ Dày Tấm Bottom Thickness</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t xml:space="preserve">8</t>
+          <t xml:space="preserve">definition:eqgyit1tf1</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t xml:space="preserve">18.6</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">10</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">18.6</t>
-        </is>
-      </c>
+          <t xml:space="preserve">definition:erhqw_82nd</t>
+        </is>
+      </c>
+      <c r="E22"/>
+      <c r="F22"/>
       <c r="G22" t="inlineStr">
         <is>
-          <t xml:space="preserve">11</t>
-        </is>
-      </c>
-      <c r="H22"/>
+          <t xml:space="preserve">length</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
       <c r="I22"/>
-      <c r="J22"/>
-      <c r="K22"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t xml:space="preserve">PLY.AC.VERKTSOI</t>
+          <t xml:space="preserve">Ngăn Kéo Ray Âm 450</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t xml:space="preserve">18.6</t>
+          <t xml:space="preserve">Panel: Độ Dày Tấm Panel Thickness | Hậu: Đáy - Độ Dày Tấm Bottom Thickness</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t xml:space="preserve">11</t>
+          <t xml:space="preserve">definition:eqgyit1tf1</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t xml:space="preserve">18.6</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">8</t>
-        </is>
-      </c>
+          <t xml:space="preserve">definition:erhqw_82nd</t>
+        </is>
+      </c>
+      <c r="E23"/>
       <c r="F23"/>
-      <c r="G23"/>
-      <c r="H23"/>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">length</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
       <c r="I23"/>
-      <c r="J23"/>
-      <c r="K23"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t xml:space="preserve">PLY.AC.VERSOI</t>
+          <t xml:space="preserve">Ngăn Kéo Ray Âm 400</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t xml:space="preserve">18.6</t>
+          <t xml:space="preserve">Panel: Độ Dày Tấm Panel Thickness | Hậu: Đáy - Độ Dày Tấm Bottom Thickness</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t xml:space="preserve">8</t>
+          <t xml:space="preserve">definition:eqgyit1tf1</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t xml:space="preserve">18.6</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t xml:space="preserve">10</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t xml:space="preserve">18.6</t>
-        </is>
-      </c>
+          <t xml:space="preserve">definition:erhqw_82nd</t>
+        </is>
+      </c>
+      <c r="E24"/>
+      <c r="F24"/>
       <c r="G24" t="inlineStr">
         <is>
-          <t xml:space="preserve">11</t>
-        </is>
-      </c>
-      <c r="H24"/>
+          <t xml:space="preserve">length</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
       <c r="I24"/>
-      <c r="J24"/>
-      <c r="K24"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t xml:space="preserve">PLY.LK</t>
+          <t xml:space="preserve">Ngăn Kéo Ray Âm 350</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t xml:space="preserve">18.6</t>
+          <t xml:space="preserve">Panel: Độ Dày Tấm Panel Thickness | Hậu: Đáy - Độ Dày Tấm Bottom Thickness</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t xml:space="preserve">11</t>
+          <t xml:space="preserve">definition:eqgyit1tf1</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t xml:space="preserve">18.6</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">10</t>
-        </is>
-      </c>
+          <t xml:space="preserve">definition:erhqw_82nd</t>
+        </is>
+      </c>
+      <c r="E25"/>
       <c r="F25"/>
-      <c r="G25"/>
-      <c r="H25"/>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">length</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
       <c r="I25"/>
-      <c r="J25"/>
-      <c r="K25"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t xml:space="preserve">PLY.VANDA</t>
+          <t xml:space="preserve">Ngăn Kéo Ray Âm 300</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t xml:space="preserve">18.6</t>
+          <t xml:space="preserve">Panel: Độ Dày Tấm Panel Thickness | Hậu: Đáy - Độ Dày Tấm Bottom Thickness</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t xml:space="preserve">11</t>
+          <t xml:space="preserve">definition:eqgyit1tf1</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t xml:space="preserve">18.6</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">18.6</t>
-        </is>
-      </c>
+          <t xml:space="preserve">definition:erhqw_82nd</t>
+        </is>
+      </c>
+      <c r="E26"/>
       <c r="F26"/>
-      <c r="G26"/>
-      <c r="H26"/>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">length</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
       <c r="I26"/>
-      <c r="J26"/>
-      <c r="K26"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t xml:space="preserve">TANBI</t>
+          <t xml:space="preserve">Ngăn Kéo Ray Âm 250</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t xml:space="preserve">20</t>
-        </is>
-      </c>
-      <c r="C27"/>
+          <t xml:space="preserve">Panel: Độ Dày Tấm Panel Thickness | Hậu: Đáy - Độ Dày Tấm Bottom Thickness</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">definition:eqgyit1tf1</t>
+        </is>
+      </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t xml:space="preserve">26</t>
+          <t xml:space="preserve">definition:erhqw_82nd</t>
         </is>
       </c>
       <c r="E27"/>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t xml:space="preserve">36</t>
-        </is>
-      </c>
-      <c r="G27"/>
+      <c r="F27"/>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">length</t>
+        </is>
+      </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t xml:space="preserve">50</t>
+          <t xml:space="preserve">1</t>
         </is>
       </c>
       <c r="I27"/>
-      <c r="J27"/>
-      <c r="K27"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t xml:space="preserve">WPB</t>
+          <t xml:space="preserve">Khung Bếp Dưới</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t xml:space="preserve">17.6</t>
+          <t xml:space="preserve">Panel: VÁN DÀY | Hậu: HẬU DÀY</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t xml:space="preserve">11</t>
+          <t xml:space="preserve">definition:dayvan</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t xml:space="preserve">17.6</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">8</t>
-        </is>
-      </c>
+          <t xml:space="preserve">definition:hauday</t>
+        </is>
+      </c>
+      <c r="E28"/>
       <c r="F28"/>
-      <c r="G28"/>
-      <c r="H28"/>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">length</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
       <c r="I28"/>
-      <c r="J28"/>
-      <c r="K28"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t xml:space="preserve">WPB.LK</t>
+          <t xml:space="preserve">khungket</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t xml:space="preserve">19.6</t>
+          <t xml:space="preserve">dodaytam</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t xml:space="preserve">11</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t xml:space="preserve">19.6</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t xml:space="preserve">8</t>
-        </is>
-      </c>
+          <t xml:space="preserve">definition:dodaytam</t>
+        </is>
+      </c>
+      <c r="D29"/>
+      <c r="E29"/>
       <c r="F29"/>
-      <c r="G29"/>
-      <c r="H29"/>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">length</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
       <c r="I29"/>
-      <c r="J29"/>
-      <c r="K29"/>
     </row>
   </sheetData>
 </worksheet>
@@ -3898,970 +4190,39 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t xml:space="preserve">match</t>
+          <t xml:space="preserve">profile_id</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t xml:space="preserve">label</t>
+          <t xml:space="preserve">profile_name</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t xml:space="preserve">param_panel</t>
+          <t xml:space="preserve">material_code</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t xml:space="preserve">param_back</t>
+          <t xml:space="preserve">panel_thickness_mm</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t xml:space="preserve">param_extra</t>
+          <t xml:space="preserve">back_thickness_mm</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t xml:space="preserve">product_only</t>
+          <t xml:space="preserve">panel_material</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t xml:space="preserve">unit</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">enabled</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">modul_only</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Tấm fix</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Độ dày</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">definition:d1</t>
-        </is>
-      </c>
-      <c r="D2"/>
-      <c r="E2"/>
-      <c r="F2"/>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">mm</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1</t>
-        </is>
-      </c>
-      <c r="I2"/>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ngắn Kéo Đáy Lùa</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Panel: Độ Dày Tấm Panel Thickness | Hậu: Đáy - Độ Dày Tấm Bottom Thickness</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">definition:eqgyit1tf1</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">definition:erhqw_82nd</t>
-        </is>
-      </c>
-      <c r="E3"/>
-      <c r="F3"/>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">mm</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1</t>
-        </is>
-      </c>
-      <c r="I3"/>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Khung Tủ Lạnh</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Độ Dày Tấm Panel Thickness, Hậu Độ Dày Tấm Back Thickness</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">definition:ba4ulq2qnw, definition:ikqikbwfw7</t>
-        </is>
-      </c>
-      <c r="D4"/>
-      <c r="E4"/>
-      <c r="F4"/>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">mm</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Khung Nóc Lọt</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Panel: Độ Dày Tấm Panel Thickness | Hậu: Hậu Độ Dày Tấm Back Thickness</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">definition:ba4ulq2qnw</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">definition:ikqikbwfw7</t>
-        </is>
-      </c>
-      <c r="E5"/>
-      <c r="F5"/>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">mm</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Khung Bếp 1</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Panel: Độ Dày Tấm Panel Thickness | Hậu: Hậu Độ Dày Tấm Back Thickness</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">definition:abh13iq2kv</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">definition:g3dnsrlh5l</t>
-        </is>
-      </c>
-      <c r="E6"/>
-      <c r="F6"/>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">length</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ngăn kéo ray bi</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Panel: Độ Dày Tấm Panel Thickness | Hậu: Đáy - Độ Dày Tấm Bottom Thickness</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">definition:eqgyit1tf1</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">definition:erhqw_82nd</t>
-        </is>
-      </c>
-      <c r="E7"/>
-      <c r="F7"/>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">mm</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1</t>
-        </is>
-      </c>
-      <c r="I7"/>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Đáy</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Chiều dày ván</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">definition:d1</t>
-        </is>
-      </c>
-      <c r="D8"/>
-      <c r="E8"/>
-      <c r="F8"/>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">mm</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1</t>
-        </is>
-      </c>
-      <c r="I8"/>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Nẹp Bù Trái 17</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Độ dày tấm</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">definition:d1</t>
-        </is>
-      </c>
-      <c r="D9"/>
-      <c r="E9"/>
-      <c r="F9"/>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">mm</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1</t>
-        </is>
-      </c>
-      <c r="I9"/>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Nẹp Bù Phải 17</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Độ dày tấm</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">definition:d1</t>
-        </is>
-      </c>
-      <c r="D10"/>
-      <c r="E10"/>
-      <c r="F10"/>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">mm</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1</t>
-        </is>
-      </c>
-      <c r="I10"/>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Nẹp Bù Phải 50</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Độ Dày Tấm</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">definition:dodaytam</t>
-        </is>
-      </c>
-      <c r="D11"/>
-      <c r="E11"/>
-      <c r="F11"/>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">mm</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1</t>
-        </is>
-      </c>
-      <c r="I11"/>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Nẹp Bù Trái 50</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Độ Dày Tấm</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">definition:dodaytam</t>
-        </is>
-      </c>
-      <c r="D12"/>
-      <c r="E12"/>
-      <c r="F12"/>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">mm</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1</t>
-        </is>
-      </c>
-      <c r="I12"/>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Đợt Cố Định</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Chiều dày ván</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">definition:d1</t>
-        </is>
-      </c>
-      <c r="D13"/>
-      <c r="E13"/>
-      <c r="F13"/>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">mm</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1</t>
-        </is>
-      </c>
-      <c r="I13"/>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Khung lavabo 1</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Độ Dày Tấm Panel Thickness, Hậu Độ Dày Tấm Back Thickness</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">definition:ba4ulq2qnw, definition:ikqikbwfw7</t>
-        </is>
-      </c>
-      <c r="D14"/>
-      <c r="E14"/>
-      <c r="F14"/>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">mm</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1</t>
-        </is>
-      </c>
-      <c r="I14"/>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Phào Nóc</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Độ Dày Tấm</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">definition:ddaytam</t>
-        </is>
-      </c>
-      <c r="D15"/>
-      <c r="E15"/>
-      <c r="F15"/>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">mm</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1</t>
-        </is>
-      </c>
-      <c r="I15"/>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ngăn Kéo Ray Âm</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Panel: Độ Dày Tấm Panel Thickness | Hậu: Đáy - Độ Dày Tấm Bottom Thickness</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">definition:eqgyit1tf1</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">definition:erhqw_82nd</t>
-        </is>
-      </c>
-      <c r="E16"/>
-      <c r="F16"/>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">mm</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1</t>
-        </is>
-      </c>
-      <c r="I16"/>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Cánh Pano</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Panel: Độ Dày Ván | Hậu: Chiều Rộng Rãnh Soi</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">definition:a0van</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">definition:c1</t>
-        </is>
-      </c>
-      <c r="E17"/>
-      <c r="F17"/>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">mm</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1</t>
-        </is>
-      </c>
-      <c r="I17"/>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Khung Nóc Phủ</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Panel: Độ Dày Tấm Panel Thickness | Hậu: Hậu Độ Dày Tấm Back Thickness</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">definition:blcep_e9zm</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">definition:j3vpfsl6fq</t>
-        </is>
-      </c>
-      <c r="E18"/>
-      <c r="F18"/>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">length</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Khung Nóc Phủ 100</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Panel: Độ Dày Tấm Panel Thickness | Hậu: Hậu Độ Dày Tấm Back Thickness</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">definition:blcep_e9zm</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">definition:j3vpfsl6fq</t>
-        </is>
-      </c>
-      <c r="E19"/>
-      <c r="F19"/>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">length</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1</t>
-        </is>
-      </c>
-      <c r="I19"/>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Chân Bệ</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">độ dày ván</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">definition:a5dodayvan</t>
-        </is>
-      </c>
-      <c r="D20"/>
-      <c r="E20"/>
-      <c r="F20"/>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">mm</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1</t>
-        </is>
-      </c>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ngăn Kéo Ray Âm 550</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Panel: Độ Dày Tấm Panel Thickness | Hậu: Đáy - Độ Dày Tấm Bottom Thickness</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">definition:eqgyit1tf1</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">definition:erhqw_82nd</t>
-        </is>
-      </c>
-      <c r="E21"/>
-      <c r="F21"/>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">length</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1</t>
-        </is>
-      </c>
-      <c r="I21"/>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ngăn Kéo Ray Âm 500</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Panel: Độ Dày Tấm Panel Thickness | Hậu: Đáy - Độ Dày Tấm Bottom Thickness</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">definition:eqgyit1tf1</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">definition:erhqw_82nd</t>
-        </is>
-      </c>
-      <c r="E22"/>
-      <c r="F22"/>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">length</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1</t>
-        </is>
-      </c>
-      <c r="I22"/>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ngăn Kéo Ray Âm 450</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Panel: Độ Dày Tấm Panel Thickness | Hậu: Đáy - Độ Dày Tấm Bottom Thickness</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">definition:eqgyit1tf1</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">definition:erhqw_82nd</t>
-        </is>
-      </c>
-      <c r="E23"/>
-      <c r="F23"/>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">length</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1</t>
-        </is>
-      </c>
-      <c r="I23"/>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ngăn Kéo Ray Âm 400</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Panel: Độ Dày Tấm Panel Thickness | Hậu: Đáy - Độ Dày Tấm Bottom Thickness</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t xml:space="preserve">definition:eqgyit1tf1</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t xml:space="preserve">definition:erhqw_82nd</t>
-        </is>
-      </c>
-      <c r="E24"/>
-      <c r="F24"/>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t xml:space="preserve">length</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1</t>
-        </is>
-      </c>
-      <c r="I24"/>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ngăn Kéo Ray Âm 350</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Panel: Độ Dày Tấm Panel Thickness | Hậu: Đáy - Độ Dày Tấm Bottom Thickness</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">definition:eqgyit1tf1</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">definition:erhqw_82nd</t>
-        </is>
-      </c>
-      <c r="E25"/>
-      <c r="F25"/>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">length</t>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1</t>
-        </is>
-      </c>
-      <c r="I25"/>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ngăn Kéo Ray Âm 300</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Panel: Độ Dày Tấm Panel Thickness | Hậu: Đáy - Độ Dày Tấm Bottom Thickness</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">definition:eqgyit1tf1</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">definition:erhqw_82nd</t>
-        </is>
-      </c>
-      <c r="E26"/>
-      <c r="F26"/>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">length</t>
-        </is>
-      </c>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1</t>
-        </is>
-      </c>
-      <c r="I26"/>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ngăn Kéo Ray Âm 250</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Panel: Độ Dày Tấm Panel Thickness | Hậu: Đáy - Độ Dày Tấm Bottom Thickness</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t xml:space="preserve">definition:eqgyit1tf1</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t xml:space="preserve">definition:erhqw_82nd</t>
-        </is>
-      </c>
-      <c r="E27"/>
-      <c r="F27"/>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t xml:space="preserve">length</t>
-        </is>
-      </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1</t>
-        </is>
-      </c>
-      <c r="I27"/>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Khung Bếp Dưới</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Panel: VÁN DÀY | Hậu: HẬU DÀY</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">definition:dayvan</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">definition:hauday</t>
-        </is>
-      </c>
-      <c r="E28"/>
-      <c r="F28"/>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">length</t>
-        </is>
-      </c>
-      <c r="H28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1</t>
-        </is>
-      </c>
-      <c r="I28"/>
+          <t xml:space="preserve">back_material</t>
+        </is>
+      </c>
     </row>
   </sheetData>
 </worksheet>
@@ -4873,39 +4234,86 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t xml:space="preserve">profile_id</t>
+          <t xml:space="preserve">enabled</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t xml:space="preserve">profile_name</t>
+          <t xml:space="preserve">material_code</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t xml:space="preserve">material_code</t>
+          <t xml:space="preserve">panel_thickness_mm</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t xml:space="preserve">panel_thickness_mm</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
           <t xml:space="preserve">back_thickness_mm</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">panel_material</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">back_material</t>
-        </is>
-      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PLY.AC.30YY-68/024-30</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">17.6</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PLY.AC.30YY-68/024-30</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">17.6</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">11</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GOSOI</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">20</t>
+        </is>
+      </c>
+      <c r="D4"/>
     </row>
   </sheetData>
 </worksheet>
@@ -4917,97 +4325,6 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t xml:space="preserve">enabled</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">material_code</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">panel_thickness_mm</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">back_thickness_mm</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PLY.AC.30YY-68/024-30</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">17.6</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">8</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PLY.AC.30YY-68/024-30</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">17.6</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">11</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">GOSOI</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">20</t>
-        </is>
-      </c>
-      <c r="D4"/>
-    </row>
-  </sheetData>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
           <t xml:space="preserve">material_name</t>
         </is>
       </c>

</xml_diff>